<commit_message>
ライセンスをApache License Version 2.0へ変更
</commit_message>
<xml_diff>
--- a/collect/manual/CSVPP_Setup_and_Usage.xlsx
+++ b/collect/manual/CSVPP_Setup_and_Usage.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="はじめに" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="314">
   <si>
     <t xml:space="preserve">はじめに</t>
   </si>
@@ -111,7 +111,7 @@
     <t xml:space="preserve">ライセンス</t>
   </si>
   <si>
-    <t xml:space="preserve">プログラム及び、ドキュメントは GNU General Public License version 2.0 のライセンスに従います。</t>
+    <t xml:space="preserve">プログラム及び、ドキュメントは Apache License Version 2.0 のライセンスに従います。</t>
   </si>
   <si>
     <t xml:space="preserve">初期設定</t>
@@ -978,6 +978,9 @@
   </si>
   <si>
     <t xml:space="preserve">マニュアルの修正</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ライセンスを Apache License Version 2.0 に変更</t>
   </si>
 </sst>
 </file>
@@ -989,7 +992,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="yyyy\年mm\月dd\日"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -1063,6 +1066,12 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1116,28 +1125,28 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1149,31 +1158,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1205,9 +1218,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>340560</xdr:colOff>
+      <xdr:colOff>339120</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>182160</xdr:rowOff>
+      <xdr:rowOff>181440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1220,8 +1233,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="281880" y="2480040"/>
-          <a:ext cx="2486160" cy="1743120"/>
+          <a:off x="281880" y="2561400"/>
+          <a:ext cx="2485440" cy="1742400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1243,9 +1256,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>273960</xdr:colOff>
+      <xdr:colOff>272520</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>94680</xdr:rowOff>
+      <xdr:rowOff>73800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1258,8 +1271,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="387000" y="5726520"/>
-          <a:ext cx="2314440" cy="3009960"/>
+          <a:off x="387000" y="5807880"/>
+          <a:ext cx="2313720" cy="3009240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1281,9 +1294,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>613440</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>10440</xdr:rowOff>
+      <xdr:colOff>612720</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>189360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1296,8 +1309,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1374120" y="6661440"/>
-          <a:ext cx="1666800" cy="2990880"/>
+          <a:off x="1374840" y="6742440"/>
+          <a:ext cx="1666080" cy="2990160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1319,9 +1332,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>415080</xdr:colOff>
+      <xdr:colOff>413640</xdr:colOff>
       <xdr:row>88</xdr:row>
-      <xdr:rowOff>16200</xdr:rowOff>
+      <xdr:rowOff>15480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1334,8 +1347,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="308160" y="10933920"/>
-          <a:ext cx="8821080" cy="6725160"/>
+          <a:off x="308160" y="11035440"/>
+          <a:ext cx="8820360" cy="6724440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1357,9 +1370,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>518400</xdr:colOff>
+      <xdr:colOff>516960</xdr:colOff>
       <xdr:row>102</xdr:row>
-      <xdr:rowOff>36720</xdr:rowOff>
+      <xdr:rowOff>36000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1372,8 +1385,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="478800" y="19108440"/>
-          <a:ext cx="2467080" cy="1371600"/>
+          <a:off x="478800" y="19209960"/>
+          <a:ext cx="2466360" cy="1370880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1395,9 +1408,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>459720</xdr:colOff>
+      <xdr:colOff>459000</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>65160</xdr:rowOff>
+      <xdr:rowOff>64440</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1406,8 +1419,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1663200" y="7507080"/>
-          <a:ext cx="595440" cy="199800"/>
+          <a:off x="1663920" y="7608600"/>
+          <a:ext cx="594720" cy="199080"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -1440,9 +1453,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>91800</xdr:colOff>
+      <xdr:colOff>91080</xdr:colOff>
       <xdr:row>88</xdr:row>
-      <xdr:rowOff>104760</xdr:rowOff>
+      <xdr:rowOff>104040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1451,8 +1464,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1485720" y="17321760"/>
-          <a:ext cx="1033560" cy="425880"/>
+          <a:off x="1486440" y="17423280"/>
+          <a:ext cx="1032840" cy="425160"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -1480,14 +1493,14 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>302400</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>46800</xdr:rowOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>145440</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>92880</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>35280</xdr:rowOff>
+      <xdr:colOff>92160</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>132840</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1496,8 +1509,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4615920" y="13089240"/>
-          <a:ext cx="419040" cy="188280"/>
+          <a:off x="4616640" y="13089240"/>
+          <a:ext cx="418320" cy="187560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1524,13 +1537,13 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>93240</xdr:colOff>
       <xdr:row>65</xdr:row>
-      <xdr:rowOff>141120</xdr:rowOff>
+      <xdr:rowOff>39600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>558720</xdr:colOff>
       <xdr:row>65</xdr:row>
-      <xdr:rowOff>141120</xdr:rowOff>
+      <xdr:rowOff>39600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1539,7 +1552,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5035320" y="13183560"/>
+          <a:off x="5036040" y="13183560"/>
           <a:ext cx="4866120" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -1574,9 +1587,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>304200</xdr:colOff>
+      <xdr:colOff>303480</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>8640</xdr:rowOff>
+      <xdr:rowOff>7920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1590,7 +1603,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="395640" y="1285920"/>
-          <a:ext cx="2494440" cy="1769400"/>
+          <a:ext cx="2493720" cy="1768680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1612,9 +1625,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>237960</xdr:colOff>
+      <xdr:colOff>237240</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>134280</xdr:rowOff>
+      <xdr:rowOff>133560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1628,7 +1641,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="500760" y="4532400"/>
-          <a:ext cx="2323080" cy="3049200"/>
+          <a:ext cx="2322360" cy="3048480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1650,9 +1663,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>259200</xdr:colOff>
+      <xdr:colOff>258480</xdr:colOff>
       <xdr:row>42</xdr:row>
-      <xdr:rowOff>50040</xdr:rowOff>
+      <xdr:rowOff>49320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1666,7 +1679,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1173240" y="5466960"/>
-          <a:ext cx="1671840" cy="3030480"/>
+          <a:ext cx="1671120" cy="3029760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1688,9 +1701,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>276120</xdr:colOff>
+      <xdr:colOff>275400</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>122400</xdr:rowOff>
+      <xdr:rowOff>121680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1700,7 +1713,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1414080" y="6113880"/>
-          <a:ext cx="801360" cy="255600"/>
+          <a:ext cx="800640" cy="254880"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -1733,9 +1746,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>300960</xdr:colOff>
+      <xdr:colOff>300240</xdr:colOff>
       <xdr:row>87</xdr:row>
-      <xdr:rowOff>29520</xdr:rowOff>
+      <xdr:rowOff>28800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1749,7 +1762,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="361440" y="9723960"/>
-          <a:ext cx="7696800" cy="7754040"/>
+          <a:ext cx="7696080" cy="7753320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1776,9 +1789,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>52200</xdr:colOff>
+      <xdr:colOff>51480</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>8280</xdr:rowOff>
+      <xdr:rowOff>7560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1791,8 +1804,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="474480" y="885600"/>
-          <a:ext cx="2494440" cy="1769400"/>
+          <a:off x="474840" y="885600"/>
+          <a:ext cx="2493720" cy="1768680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1814,9 +1827,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>428760</xdr:colOff>
+      <xdr:colOff>427680</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>9360</xdr:rowOff>
+      <xdr:rowOff>8640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1829,8 +1842,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="402120" y="4646880"/>
-          <a:ext cx="2314440" cy="3009960"/>
+          <a:off x="402480" y="4646880"/>
+          <a:ext cx="2313720" cy="3009240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1852,9 +1865,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>165600</xdr:colOff>
+      <xdr:colOff>165240</xdr:colOff>
       <xdr:row>42</xdr:row>
-      <xdr:rowOff>110160</xdr:rowOff>
+      <xdr:rowOff>109440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1867,8 +1880,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1415520" y="5566680"/>
-          <a:ext cx="1666800" cy="2990880"/>
+          <a:off x="1416240" y="5566680"/>
+          <a:ext cx="1666080" cy="2990160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1890,9 +1903,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>627480</xdr:colOff>
+      <xdr:colOff>626760</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>174600</xdr:rowOff>
+      <xdr:rowOff>173880</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1901,8 +1914,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1658520" y="6024960"/>
-          <a:ext cx="628200" cy="196920"/>
+          <a:off x="1659240" y="6024960"/>
+          <a:ext cx="627480" cy="196200"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -1935,9 +1948,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>610560</xdr:colOff>
+      <xdr:colOff>609840</xdr:colOff>
       <xdr:row>69</xdr:row>
-      <xdr:rowOff>66960</xdr:rowOff>
+      <xdr:rowOff>66240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1950,8 +1963,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="421200" y="9333360"/>
-          <a:ext cx="8135280" cy="4581720"/>
+          <a:off x="421560" y="9333360"/>
+          <a:ext cx="8134560" cy="4581000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1973,9 +1986,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>523800</xdr:colOff>
+      <xdr:colOff>522720</xdr:colOff>
       <xdr:row>85</xdr:row>
-      <xdr:rowOff>66600</xdr:rowOff>
+      <xdr:rowOff>65880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1988,8 +2001,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="449640" y="15448320"/>
-          <a:ext cx="1733400" cy="1666800"/>
+          <a:off x="450000" y="15448320"/>
+          <a:ext cx="1732680" cy="1666080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2011,9 +2024,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>428760</xdr:colOff>
+      <xdr:colOff>427680</xdr:colOff>
       <xdr:row>102</xdr:row>
-      <xdr:rowOff>199800</xdr:rowOff>
+      <xdr:rowOff>199080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2026,8 +2039,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="402120" y="17638920"/>
-          <a:ext cx="2314440" cy="3009960"/>
+          <a:off x="402480" y="17638920"/>
+          <a:ext cx="2313720" cy="3009240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2049,9 +2062,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>485640</xdr:colOff>
+      <xdr:colOff>485280</xdr:colOff>
       <xdr:row>106</xdr:row>
-      <xdr:rowOff>47880</xdr:rowOff>
+      <xdr:rowOff>47160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2064,8 +2077,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1735560" y="18306000"/>
-          <a:ext cx="1666800" cy="2990880"/>
+          <a:off x="1736280" y="18306000"/>
+          <a:ext cx="1666080" cy="2990160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2087,9 +2100,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>307080</xdr:colOff>
+      <xdr:colOff>306360</xdr:colOff>
       <xdr:row>93</xdr:row>
-      <xdr:rowOff>101520</xdr:rowOff>
+      <xdr:rowOff>100800</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2098,8 +2111,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2002320" y="18553320"/>
-          <a:ext cx="592560" cy="196920"/>
+          <a:off x="2003040" y="18553320"/>
+          <a:ext cx="591840" cy="196200"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -2132,9 +2145,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>304560</xdr:colOff>
+      <xdr:colOff>303480</xdr:colOff>
       <xdr:row>152</xdr:row>
-      <xdr:rowOff>115200</xdr:rowOff>
+      <xdr:rowOff>114480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2147,8 +2160,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="402120" y="23849280"/>
-          <a:ext cx="8476920" cy="6716160"/>
+          <a:off x="402480" y="23849280"/>
+          <a:ext cx="8476200" cy="6715440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2170,9 +2183,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>313920</xdr:colOff>
+      <xdr:colOff>313200</xdr:colOff>
       <xdr:row>132</xdr:row>
-      <xdr:rowOff>94680</xdr:rowOff>
+      <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2181,8 +2194,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1364040" y="26316360"/>
-          <a:ext cx="1237680" cy="227880"/>
+          <a:off x="1364760" y="26316360"/>
+          <a:ext cx="1236960" cy="227160"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -2215,9 +2228,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>563040</xdr:colOff>
+      <xdr:colOff>562320</xdr:colOff>
       <xdr:row>192</xdr:row>
-      <xdr:rowOff>181440</xdr:rowOff>
+      <xdr:rowOff>180720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2230,8 +2243,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="402120" y="32650560"/>
-          <a:ext cx="10621440" cy="5982120"/>
+          <a:off x="402480" y="32650560"/>
+          <a:ext cx="10620720" cy="5981400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2253,9 +2266,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>591480</xdr:colOff>
+      <xdr:colOff>590760</xdr:colOff>
       <xdr:row>219</xdr:row>
-      <xdr:rowOff>181080</xdr:rowOff>
+      <xdr:rowOff>180360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2268,8 +2281,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="402120" y="39451320"/>
-          <a:ext cx="8135280" cy="4581720"/>
+          <a:off x="402480" y="39451320"/>
+          <a:ext cx="8134560" cy="4581000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2291,9 +2304,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>190080</xdr:colOff>
+      <xdr:colOff>189360</xdr:colOff>
       <xdr:row>206</xdr:row>
-      <xdr:rowOff>161640</xdr:rowOff>
+      <xdr:rowOff>160920</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2302,8 +2315,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="402120" y="41194440"/>
-          <a:ext cx="2704680" cy="218880"/>
+          <a:off x="402480" y="41194440"/>
+          <a:ext cx="2703960" cy="218160"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -2341,9 +2354,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>180720</xdr:colOff>
+      <xdr:colOff>180000</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>190440</xdr:rowOff>
+      <xdr:rowOff>189720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2356,8 +2369,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4581360" y="2027520"/>
-          <a:ext cx="2314440" cy="3009960"/>
+          <a:off x="4583160" y="2027520"/>
+          <a:ext cx="2313720" cy="3009240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2379,9 +2392,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>199800</xdr:colOff>
+      <xdr:colOff>199080</xdr:colOff>
       <xdr:row>42</xdr:row>
-      <xdr:rowOff>152640</xdr:rowOff>
+      <xdr:rowOff>151920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2394,8 +2407,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4619520" y="5609160"/>
-          <a:ext cx="1666800" cy="2990880"/>
+          <a:off x="4621320" y="5609160"/>
+          <a:ext cx="1666080" cy="2990160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2932,7 +2945,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="3" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>30</v>
@@ -2946,7 +2959,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" s="3" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="2" t="s">
         <v>31</v>
@@ -2960,7 +2973,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" s="3" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="2" t="s">
         <v>32</v>
@@ -2974,7 +2987,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="3" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
@@ -3032,7 +3045,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" s="3" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -3440,7 +3453,7 @@
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="17.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="17.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="38.13"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="2" width="9"/>
   </cols>
@@ -3792,7 +3805,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="9" width="9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
         <v>162</v>
       </c>
@@ -4640,8 +4653,19 @@
         <v>312</v>
       </c>
     </row>
+    <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="B80" s="13" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C80" s="15" t="s">
+        <v>313</v>
+      </c>
+    </row>
     <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="15"/>
+      <c r="A81" s="16"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>